<commit_message>
JO: apply Centrifugal Blower beautification to Centrifugal Inline
Concatenate the composite lines, center on the underline, color the five secondary
values red, and make the (make) parenthetical red in the header — same as the
Centrifugal Blower. Pure zip-surgery (drawing/images byte-identical, underline rows
untouched); uses the Inline's own Arial fonts.
</commit_message>
<xml_diff>
--- a/public/templates/fans-inline-jo-template.xlsx
+++ b/public/templates/fans-inline-jo-template.xlsx
@@ -976,7 +976,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1202,6 +1202,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1724,6 +1730,9 @@
       <c r="B15" t="s">
         <v>18</v>
       </c>
+      <c r="C15" s="83">
+        <f>Source!B70&amp;" "&amp;Source!B71&amp;"   "&amp;Source!B77&amp;""" Ø   "&amp;Source!B67</f>
+      </c>
       <c r="F15" s="4">
         <f>Source!B70</f>
         <v>1</v>
@@ -1750,7 +1759,9 @@
       <c r="P15" s="35" t="s">
         <v>204</v>
       </c>
-      <c r="Q15" s="20"/>
+      <c r="Q15" s="84">
+        <f>"   ("&amp;Source!B68&amp;")"</f>
+      </c>
       <c r="R15" s="36" t="str">
         <f>Source!B68</f>
         <v xml:space="preserve">Standard </v>
@@ -1990,9 +2001,8 @@
       <c r="B40" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C40" s="64" t="str">
+      <c r="C40" s="83">
         <f>Source!B82</f>
-        <v>520 cfm @ 2" w.g.</v>
       </c>
       <c r="D40" s="64"/>
       <c r="E40" s="64"/>
@@ -2006,7 +2016,9 @@
         <v>1238 cfm @ 0" w.g.</v>
       </c>
       <c r="L40" s="64"/>
-      <c r="M40" s="64"/>
+      <c r="M40" s="84">
+        <f>" "&amp;Source!B83</f>
+      </c>
       <c r="N40" s="64"/>
       <c r="O40" s="64"/>
       <c r="P40" s="9"/>
@@ -2054,9 +2066,8 @@
       <c r="B42" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C42" s="64">
-        <f>Source!B84</f>
-        <v>2221</v>
+      <c r="C42" s="83">
+        <f>Source!B84&amp;" rpm"</f>
       </c>
       <c r="D42" s="60"/>
       <c r="E42" s="60"/>
@@ -2074,7 +2085,9 @@
         <v>53</v>
       </c>
       <c r="L42" s="4"/>
-      <c r="M42" s="4"/>
+      <c r="M42" s="84">
+        <f>" "&amp;ROUNDUP(Source!D76,0)&amp;" rpm"</f>
+      </c>
       <c r="N42" s="4"/>
       <c r="O42" s="4"/>
       <c r="P42" s="9"/>
@@ -2219,9 +2232,8 @@
       <c r="B46" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C46" s="67">
-        <f>Source!B96</f>
-        <v>4</v>
+      <c r="C46" s="83">
+        <f>TRIM(TEXT(Source!B96,"# ?/?"))&amp;""" Ø x "&amp;Source!D93&amp;" x "&amp;Source!D91&amp;" mm Ø bore x "&amp;Source!D92&amp;" mm keyway"</f>
       </c>
       <c r="D46" s="70"/>
       <c r="E46" s="59" t="s">
@@ -2255,7 +2267,9 @@
       <c r="P46" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="Q46" s="59"/>
+      <c r="Q46" s="84">
+        <f>" "&amp;Source!D94&amp;" mm Ø Hub"</f>
+      </c>
       <c r="R46" s="59"/>
       <c r="S46" s="4"/>
       <c r="T46" s="4"/>
@@ -2303,9 +2317,8 @@
       <c r="B48" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C48" s="67">
-        <f>Source!B97</f>
-        <v>3</v>
+      <c r="C48" s="83">
+        <f>TRIM(TEXT(Source!B97,"# ?/?"))&amp;""" Ø x "&amp;Source!D93&amp;" x "&amp;Source!D80</f>
       </c>
       <c r="D48" s="67"/>
       <c r="E48" s="59" t="s">
@@ -2330,7 +2343,9 @@
       <c r="N48" s="63"/>
       <c r="O48" s="63"/>
       <c r="P48" s="63"/>
-      <c r="Q48" s="63"/>
+      <c r="Q48" s="84">
+        <f>" "&amp;Source!D95&amp;" mm Ø Hub"</f>
+      </c>
       <c r="R48" s="63"/>
       <c r="S48" s="4"/>
       <c r="T48" s="4"/>
@@ -2558,9 +2573,8 @@
       <c r="B56" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C56" s="59" t="str">
-        <f>Source!D78</f>
-        <v>UCF205</v>
+      <c r="C56" s="83">
+        <f>Source!D78&amp;"  --"</f>
       </c>
       <c r="D56" s="59"/>
       <c r="E56" s="59"/>
@@ -2578,7 +2592,9 @@
       <c r="L56" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="M56" s="4"/>
+      <c r="M56" s="84">
+        <f>" "&amp;SUM(Source!B70)*2&amp;" pcs"</f>
+      </c>
       <c r="N56" s="4"/>
       <c r="O56" s="4"/>
       <c r="P56" s="4"/>
@@ -2633,42 +2649,38 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <mergeCells count="35">
+  <mergeCells count="31">
     <mergeCell ref="A12:W12"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="L20:M20"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="E48:F48"/>
     <mergeCell ref="O36:P36"/>
     <mergeCell ref="C36:N36"/>
     <mergeCell ref="C38:N38"/>
-    <mergeCell ref="J48:R48"/>
-    <mergeCell ref="G48:H48"/>
     <mergeCell ref="R36:V36"/>
     <mergeCell ref="R38:V38"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="K46:M46"/>
-    <mergeCell ref="P46:R46"/>
     <mergeCell ref="G44:H44"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="G46:H46"/>
     <mergeCell ref="S58:W58"/>
     <mergeCell ref="D13:K13"/>
     <mergeCell ref="S13:V13"/>
-    <mergeCell ref="H15:I15"/>
     <mergeCell ref="C17:G17"/>
-    <mergeCell ref="C56:F56"/>
     <mergeCell ref="C54:I54"/>
     <mergeCell ref="D52:M52"/>
     <mergeCell ref="C50:P50"/>
     <mergeCell ref="O38:P38"/>
     <mergeCell ref="P44:S44"/>
-    <mergeCell ref="C40:I40"/>
-    <mergeCell ref="K40:O40"/>
-    <mergeCell ref="C42:E42"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C15:P15"/>
+    <mergeCell ref="Q15:V15"/>
+    <mergeCell ref="C40:L40"/>
+    <mergeCell ref="M40:V40"/>
+    <mergeCell ref="C42:L42"/>
+    <mergeCell ref="M42:V42"/>
+    <mergeCell ref="C46:P46"/>
+    <mergeCell ref="Q46:V46"/>
+    <mergeCell ref="C48:P48"/>
+    <mergeCell ref="Q48:V48"/>
+    <mergeCell ref="C56:L56"/>
+    <mergeCell ref="M56:V56"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
JO: concatenate the motor spec line (row 44) on Centrifugal Inline, matching the Blower
</commit_message>
<xml_diff>
--- a/public/templates/fans-inline-jo-template.xlsx
+++ b/public/templates/fans-inline-jo-template.xlsx
@@ -2135,9 +2135,8 @@
       <c r="B44" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C44" s="41">
-        <f>Source!D87</f>
-        <v>3</v>
+      <c r="C44" s="83">
+        <f>TRIM(TEXT(Source!D87,"# ?/?"))&amp;" HP,  "&amp;Source!D88&amp;" PH,  "&amp;Source!B90&amp;" V,  "&amp;Source!B91&amp;" Hz,  "&amp;Source!D90&amp;" pole,  "&amp;Source!D89&amp;" rpm,  "&amp;Source!B92&amp;",  "&amp;Source!B87&amp;",  "&amp;Source!B93</f>
       </c>
       <c r="D44" s="3" t="s">
         <v>63</v>
@@ -2649,7 +2648,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <mergeCells count="31">
+  <mergeCells count="30">
     <mergeCell ref="A12:W12"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="H20:I20"/>
@@ -2659,7 +2658,6 @@
     <mergeCell ref="C38:N38"/>
     <mergeCell ref="R36:V36"/>
     <mergeCell ref="R38:V38"/>
-    <mergeCell ref="G44:H44"/>
     <mergeCell ref="S58:W58"/>
     <mergeCell ref="D13:K13"/>
     <mergeCell ref="S13:V13"/>
@@ -2668,7 +2666,6 @@
     <mergeCell ref="D52:M52"/>
     <mergeCell ref="C50:P50"/>
     <mergeCell ref="O38:P38"/>
-    <mergeCell ref="P44:S44"/>
     <mergeCell ref="C15:P15"/>
     <mergeCell ref="Q15:V15"/>
     <mergeCell ref="C40:L40"/>
@@ -2681,6 +2678,7 @@
     <mergeCell ref="Q48:V48"/>
     <mergeCell ref="C56:L56"/>
     <mergeCell ref="M56:V56"/>
+    <mergeCell ref="C44:V44"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>